<commit_message>
feat: staffing import, chat tools, memory, and auto titles
Ship daily staffing with stints/summary, chat staffing tool, conversation memory, and rule+LLM titles; harden Milvus ACL (kb_chunks_v5) and archive completed OpenSpec changes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/v1模型选型与预算.xlsx
+++ b/docs/v1模型选型与预算.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255"/>
+    <workbookView windowWidth="28800" windowHeight="11805" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="选型结论" sheetId="1" r:id="rId1"/>
@@ -1112,7 +1112,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1139,13 +1139,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1619,148 +1612,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2480,7 +2473,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" ht="27" spans="1:3">
+    <row r="16" spans="1:3">
       <c r="A16" s="3" t="s">
         <v>83</v>
       </c>

</xml_diff>